<commit_message>
Rebuild every deliverable from the reconciled warehouse
One clean pass of the whole chain -- semantic model, report, evidence pack
figures, HTML, PDF and Excel -- so that what is committed is what the scripts
produce rather than what accumulated across a session of fixes.
</commit_message>
<xml_diff>
--- a/docs/Drakens_Energy_360_Report.xlsx
+++ b/docs/Drakens_Energy_360_Report.xlsx
@@ -647,21 +647,21 @@
     <t>debit_amount_zar_non_negative</t>
   </si>
   <si>
+    <t>solar_reading_id_present</t>
+  </si>
+  <si>
     <t>order_id_present</t>
   </si>
   <si>
-    <t>solar_reading_id_present</t>
-  </si>
-  <si>
     <t>qualifying_spend_zar_non_negative</t>
   </si>
   <si>
+    <t>volume_litres_non_negative</t>
+  </si>
+  <si>
     <t>customer_id_present</t>
   </si>
   <si>
-    <t>volume_litres_non_negative</t>
-  </si>
-  <si>
     <t>credit_amount_zar_non_negative</t>
   </si>
   <si>
@@ -701,25 +701,25 @@
     <t>delivered_litres_within_range</t>
   </si>
   <si>
+    <t>work_order_id_present</t>
+  </si>
+  <si>
     <t>grid_cost_zar_non_negative</t>
   </si>
   <si>
-    <t>work_order_id_present</t>
+    <t>rated_power_kw_non_negative</t>
+  </si>
+  <si>
+    <t>labour_cost_zar_non_negative</t>
   </si>
   <si>
     <t>total_cost_zar_non_negative</t>
   </si>
   <si>
-    <t>rated_power_kw_non_negative</t>
-  </si>
-  <si>
-    <t>labour_cost_zar_non_negative</t>
+    <t>average_power_kw_non_negative</t>
   </si>
   <si>
     <t>parts_cost_zar_non_negative</t>
-  </si>
-  <si>
-    <t>average_power_kw_non_negative</t>
   </si>
   <si>
     <t>incident_id_present</t>
@@ -6404,10 +6404,10 @@
         <v>205</v>
       </c>
       <c r="B31" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C31" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D31">
         <v>88</v>
@@ -6418,10 +6418,10 @@
         <v>206</v>
       </c>
       <c r="B32" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C32" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D32">
         <v>88</v>
@@ -6614,10 +6614,10 @@
         <v>220</v>
       </c>
       <c r="B46" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C46" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D46">
         <v>8</v>
@@ -6628,10 +6628,10 @@
         <v>221</v>
       </c>
       <c r="B47" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C47" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D47">
         <v>8</v>

</xml_diff>